<commit_message>
Show academic years as 25-26 and the winter interim as WI, converting from and to the data's AY25 and Spring part 0
Assisted by Claude Sonnet 5.5 (Anthropic).
</commit_message>
<xml_diff>
--- a/apps/web/public/examples/example-merging-amus.xlsx
+++ b/apps/web/public/examples/example-merging-amus.xlsx
@@ -208,327 +208,327 @@
     <t>Added for the merging example: a second section for the first-year cohort</t>
   </si>
   <si>
+    <t>181</t>
+  </si>
+  <si>
+    <t>SP-0</t>
+  </si>
+  <si>
+    <t>Algorithms and Music</t>
+  </si>
+  <si>
+    <t>Cy Fictional</t>
+  </si>
+  <si>
+    <t>Winter intensive: meets every weekday for two weeks</t>
+  </si>
+  <si>
+    <t>203</t>
+  </si>
+  <si>
+    <t>08:00:00 - 09:05:00</t>
+  </si>
+  <si>
+    <t>NH 103</t>
+  </si>
+  <si>
+    <t>Discrete Rhythm</t>
+  </si>
+  <si>
+    <t>228</t>
+  </si>
+  <si>
+    <t>TR</t>
+  </si>
+  <si>
+    <t>10:20:00 - 12:00:00</t>
+  </si>
+  <si>
+    <t>Harmonic Structures</t>
+  </si>
+  <si>
+    <t>235</t>
+  </si>
+  <si>
+    <t>Multivoice Analysis</t>
+  </si>
+  <si>
+    <t>368</t>
+  </si>
+  <si>
+    <t>14:10:00 - 15:50:00</t>
+  </si>
+  <si>
+    <t>NH 104</t>
+  </si>
+  <si>
+    <t>Corpus Studies I</t>
+  </si>
+  <si>
+    <t>375</t>
+  </si>
+  <si>
+    <t>Corpus Studies II</t>
+  </si>
+  <si>
+    <t>SectionId</t>
+  </si>
+  <si>
+    <t>Department</t>
+  </si>
+  <si>
+    <t>AcademicYear</t>
+  </si>
+  <si>
+    <t>MinimumCredits</t>
+  </si>
+  <si>
+    <t>MaximumCredits</t>
+  </si>
+  <si>
+    <t>StartTime</t>
+  </si>
+  <si>
+    <t>MeetingDuration</t>
+  </si>
+  <si>
+    <t>Classroom</t>
+  </si>
+  <si>
+    <t>CourseLevel</t>
+  </si>
+  <si>
+    <t>Group</t>
+  </si>
+  <si>
+    <t>Enrollment</t>
+  </si>
+  <si>
+    <t>EnrollmentDay10</t>
+  </si>
+  <si>
+    <t>AY25-FA-AMUS112-A</t>
+  </si>
+  <si>
+    <t>AY25</t>
+  </si>
+  <si>
+    <t>09:15</t>
+  </si>
+  <si>
+    <t>AY25-FA-AMUS112-B</t>
+  </si>
+  <si>
+    <t>11:00</t>
+  </si>
+  <si>
+    <t>AY25-FA-AMUS145-A</t>
+  </si>
+  <si>
+    <t>12:15</t>
+  </si>
+  <si>
+    <t>AY25-FA-AMUS228-A</t>
+  </si>
+  <si>
+    <t>10:20</t>
+  </si>
+  <si>
+    <t>AY25-FA-AMUS203-A</t>
+  </si>
+  <si>
+    <t>08:00</t>
+  </si>
+  <si>
+    <t>AY25-FA-AMUS368-A</t>
+  </si>
+  <si>
+    <t>14:10</t>
+  </si>
+  <si>
+    <t>AY25-WI-AMUS181-A</t>
+  </si>
+  <si>
+    <t>09:00</t>
+  </si>
+  <si>
+    <t>AY25-SP-AMUS119-A</t>
+  </si>
+  <si>
+    <t>AY25-SP-AMUS145-A</t>
+  </si>
+  <si>
+    <t>AY25-SP-AMUS235-A</t>
+  </si>
+  <si>
+    <t>AY25-SP-AMUS375-A</t>
+  </si>
+  <si>
+    <t>AY25-SU-AMUS112-A</t>
+  </si>
+  <si>
+    <t>AY25-FA-AMUS145-B</t>
+  </si>
+  <si>
+    <t>13:30</t>
+  </si>
+  <si>
+    <t>Activity</t>
+  </si>
+  <si>
+    <t>Load</t>
+  </si>
+  <si>
+    <t>AY</t>
+  </si>
+  <si>
+    <t>Constraint</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>Course</t>
+  </si>
+  <si>
+    <t>Instructor</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
+    <t>Choose</t>
+  </si>
+  <si>
+    <t>Bound</t>
+  </si>
+  <si>
+    <t>Gap</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>Starts</t>
+  </si>
+  <si>
+    <t>Days</t>
+  </si>
+  <si>
+    <t>DayRule</t>
+  </si>
+  <si>
+    <t>From</t>
+  </si>
+  <si>
+    <t>To</t>
+  </si>
+  <si>
+    <t>Should</t>
+  </si>
+  <si>
+    <t>Meets</t>
+  </si>
+  <si>
+    <t>Element</t>
+  </si>
+  <si>
+    <t>Capacity</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Intensive terms meet daily</t>
+  </si>
+  <si>
+    <t>standard</t>
+  </si>
+  <si>
+    <t>*</t>
+  </si>
+  <si>
+    <t>WI, SU</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Winter and summer courses meet every weekday for a few hours; these times are not in the university's list.</t>
+  </si>
+  <si>
+    <t>allow</t>
+  </si>
+  <si>
+    <t>150</t>
+  </si>
+  <si>
+    <t>13:00</t>
+  </si>
+  <si>
+    <t>First-year cohort</t>
+  </si>
+  <si>
+    <t>cohortPlan</t>
+  </si>
+  <si>
+    <t>AMUS 112</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>Two groups of 30 first-year students who share BHAV 112 and DIGI 225. The courses are in three schedules, so the rule can only be checked when they are merged.</t>
+  </si>
+  <si>
+    <t>BHAV 112</t>
+  </si>
+  <si>
+    <t>DIGI 225</t>
+  </si>
+  <si>
+    <t>AMUS 145</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>Kind</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>StartWeek</t>
+  </si>
+  <si>
+    <t>EndWeek</t>
+  </si>
+  <si>
+    <t>SpreadTerm</t>
+  </si>
+  <si>
+    <t>NonRoom</t>
+  </si>
+  <si>
+    <t>Off Campus</t>
+  </si>
+  <si>
+    <t>Online</t>
+  </si>
+  <si>
+    <t>TBD</t>
+  </si>
+  <si>
+    <t>Fall</t>
+  </si>
+  <si>
     <t>WI</t>
   </si>
   <si>
-    <t>181</t>
-  </si>
-  <si>
-    <t>WI-Full</t>
-  </si>
-  <si>
-    <t>Algorithms and Music</t>
-  </si>
-  <si>
-    <t>Cy Fictional</t>
-  </si>
-  <si>
-    <t>Winter intensive: meets every weekday for two weeks</t>
-  </si>
-  <si>
-    <t>203</t>
-  </si>
-  <si>
-    <t>08:00:00 - 09:05:00</t>
-  </si>
-  <si>
-    <t>NH 103</t>
-  </si>
-  <si>
-    <t>Discrete Rhythm</t>
-  </si>
-  <si>
-    <t>228</t>
-  </si>
-  <si>
-    <t>TR</t>
-  </si>
-  <si>
-    <t>10:20:00 - 12:00:00</t>
-  </si>
-  <si>
-    <t>Harmonic Structures</t>
-  </si>
-  <si>
-    <t>235</t>
-  </si>
-  <si>
-    <t>Multivoice Analysis</t>
-  </si>
-  <si>
-    <t>368</t>
-  </si>
-  <si>
-    <t>14:10:00 - 15:50:00</t>
-  </si>
-  <si>
-    <t>NH 104</t>
-  </si>
-  <si>
-    <t>Corpus Studies I</t>
-  </si>
-  <si>
-    <t>375</t>
-  </si>
-  <si>
-    <t>Corpus Studies II</t>
-  </si>
-  <si>
-    <t>SectionId</t>
-  </si>
-  <si>
-    <t>Department</t>
-  </si>
-  <si>
-    <t>AcademicYear</t>
-  </si>
-  <si>
-    <t>MinimumCredits</t>
-  </si>
-  <si>
-    <t>MaximumCredits</t>
-  </si>
-  <si>
-    <t>StartTime</t>
-  </si>
-  <si>
-    <t>MeetingDuration</t>
-  </si>
-  <si>
-    <t>Classroom</t>
-  </si>
-  <si>
-    <t>CourseLevel</t>
-  </si>
-  <si>
-    <t>Group</t>
-  </si>
-  <si>
-    <t>Enrollment</t>
-  </si>
-  <si>
-    <t>EnrollmentDay10</t>
-  </si>
-  <si>
-    <t>AY25-FA-AMUS112-A</t>
-  </si>
-  <si>
-    <t>AY25</t>
-  </si>
-  <si>
-    <t>09:15</t>
-  </si>
-  <si>
-    <t>AY25-FA-AMUS112-B</t>
-  </si>
-  <si>
-    <t>11:00</t>
-  </si>
-  <si>
-    <t>AY25-FA-AMUS145-A</t>
-  </si>
-  <si>
-    <t>12:15</t>
-  </si>
-  <si>
-    <t>AY25-FA-AMUS228-A</t>
-  </si>
-  <si>
-    <t>10:20</t>
-  </si>
-  <si>
-    <t>AY25-FA-AMUS203-A</t>
-  </si>
-  <si>
-    <t>08:00</t>
-  </si>
-  <si>
-    <t>AY25-FA-AMUS368-A</t>
-  </si>
-  <si>
-    <t>14:10</t>
-  </si>
-  <si>
-    <t>AY25-WI-AMUS181-A</t>
-  </si>
-  <si>
-    <t>09:00</t>
-  </si>
-  <si>
-    <t>AY25-SP-AMUS119-A</t>
-  </si>
-  <si>
-    <t>AY25-SP-AMUS145-A</t>
-  </si>
-  <si>
-    <t>AY25-SP-AMUS235-A</t>
-  </si>
-  <si>
-    <t>AY25-SP-AMUS375-A</t>
-  </si>
-  <si>
-    <t>AY25-SU-AMUS112-A</t>
-  </si>
-  <si>
-    <t>AY25-FA-AMUS145-B</t>
-  </si>
-  <si>
-    <t>13:30</t>
-  </si>
-  <si>
-    <t>Activity</t>
-  </si>
-  <si>
-    <t>Load</t>
-  </si>
-  <si>
-    <t>AY</t>
-  </si>
-  <si>
-    <t>Constraint</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
-    <t>Course</t>
-  </si>
-  <si>
-    <t>Instructor</t>
-  </si>
-  <si>
-    <t>Count</t>
-  </si>
-  <si>
-    <t>Choose</t>
-  </si>
-  <si>
-    <t>Bound</t>
-  </si>
-  <si>
-    <t>Gap</t>
-  </si>
-  <si>
-    <t>Action</t>
-  </si>
-  <si>
-    <t>Starts</t>
-  </si>
-  <si>
-    <t>Days</t>
-  </si>
-  <si>
-    <t>DayRule</t>
-  </si>
-  <si>
-    <t>From</t>
-  </si>
-  <si>
-    <t>To</t>
-  </si>
-  <si>
-    <t>Should</t>
-  </si>
-  <si>
-    <t>Meets</t>
-  </si>
-  <si>
-    <t>Element</t>
-  </si>
-  <si>
-    <t>Capacity</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>Intensive terms meet daily</t>
-  </si>
-  <si>
-    <t>standard</t>
-  </si>
-  <si>
-    <t>*</t>
-  </si>
-  <si>
-    <t>WI, SU</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Winter and summer courses meet every weekday for a few hours; these times are not in the university's list.</t>
-  </si>
-  <si>
-    <t>allow</t>
-  </si>
-  <si>
-    <t>150</t>
-  </si>
-  <si>
-    <t>13:00</t>
-  </si>
-  <si>
-    <t>First-year cohort</t>
-  </si>
-  <si>
-    <t>cohortPlan</t>
-  </si>
-  <si>
-    <t>AMUS 112</t>
-  </si>
-  <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>Two groups of 30 first-year students who share BHAV 112 and DIGI 225. The courses are in three schedules, so the rule can only be checked when they are merged.</t>
-  </si>
-  <si>
-    <t>BHAV 112</t>
-  </si>
-  <si>
-    <t>DIGI 225</t>
-  </si>
-  <si>
-    <t>AMUS 145</t>
-  </si>
-  <si>
-    <t>25</t>
-  </si>
-  <si>
-    <t>Kind</t>
-  </si>
-  <si>
-    <t>Code</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>StartWeek</t>
-  </si>
-  <si>
-    <t>EndWeek</t>
-  </si>
-  <si>
-    <t>SpreadTerm</t>
-  </si>
-  <si>
-    <t>NonRoom</t>
-  </si>
-  <si>
-    <t>Off Campus</t>
-  </si>
-  <si>
-    <t>Online</t>
-  </si>
-  <si>
-    <t>TBD</t>
-  </si>
-  <si>
-    <t>Fall</t>
-  </si>
-  <si>
     <t>Winter Intensive</t>
   </si>
   <si>
@@ -592,7 +592,7 @@
     <t>Export Time</t>
   </si>
   <si>
-    <t>08:51:36</t>
+    <t>12:17:43</t>
   </si>
   <si>
     <t>Academic Year</t>
@@ -1771,13 +1771,13 @@
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="B12" t="s">
         <v>36</v>
       </c>
       <c r="C12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D12" t="s">
         <v>38</v>
@@ -1798,19 +1798,19 @@
         <v>42</v>
       </c>
       <c r="J12" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="K12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="L12">
         <v>150</v>
       </c>
       <c r="M12" t="s">
+        <v>65</v>
+      </c>
+      <c r="N12" t="s">
         <v>66</v>
-      </c>
-      <c r="N12" t="s">
-        <v>67</v>
       </c>
       <c r="O12" t="s">
         <v>44</v>
@@ -1819,7 +1819,7 @@
         <v>45</v>
       </c>
       <c r="Q12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="R12" t="s">
         <v>23</v>
@@ -1845,7 +1845,7 @@
         <v>36</v>
       </c>
       <c r="C13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D13" t="s">
         <v>38</v>
@@ -1860,10 +1860,10 @@
         <v>40</v>
       </c>
       <c r="H13" t="s">
+        <v>69</v>
+      </c>
+      <c r="I13" t="s">
         <v>70</v>
-      </c>
-      <c r="I13" t="s">
-        <v>71</v>
       </c>
       <c r="J13" t="s">
         <v>26</v>
@@ -1875,10 +1875,10 @@
         <v>65</v>
       </c>
       <c r="M13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="N13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O13" t="s">
         <v>44</v>
@@ -1913,7 +1913,7 @@
         <v>36</v>
       </c>
       <c r="C14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D14" t="s">
         <v>38</v>
@@ -1925,13 +1925,13 @@
         <v>39</v>
       </c>
       <c r="G14" t="s">
+        <v>73</v>
+      </c>
+      <c r="H14" t="s">
         <v>74</v>
       </c>
-      <c r="H14" t="s">
-        <v>75</v>
-      </c>
       <c r="I14" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J14" t="s">
         <v>26</v>
@@ -1943,10 +1943,10 @@
         <v>100</v>
       </c>
       <c r="M14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="N14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O14" t="s">
         <v>44</v>
@@ -1981,7 +1981,7 @@
         <v>36</v>
       </c>
       <c r="C15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D15" t="s">
         <v>38</v>
@@ -1993,13 +1993,13 @@
         <v>39</v>
       </c>
       <c r="G15" t="s">
+        <v>73</v>
+      </c>
+      <c r="H15" t="s">
         <v>74</v>
       </c>
-      <c r="H15" t="s">
-        <v>75</v>
-      </c>
       <c r="I15" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J15" t="s">
         <v>26</v>
@@ -2011,10 +2011,10 @@
         <v>100</v>
       </c>
       <c r="M15" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="N15" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O15" t="s">
         <v>44</v>
@@ -2049,7 +2049,7 @@
         <v>36</v>
       </c>
       <c r="C16" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D16" t="s">
         <v>38</v>
@@ -2061,13 +2061,13 @@
         <v>39</v>
       </c>
       <c r="G16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H16" t="s">
+        <v>79</v>
+      </c>
+      <c r="I16" t="s">
         <v>80</v>
-      </c>
-      <c r="I16" t="s">
-        <v>81</v>
       </c>
       <c r="J16" t="s">
         <v>26</v>
@@ -2079,7 +2079,7 @@
         <v>100</v>
       </c>
       <c r="M16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="N16" t="s">
         <v>34</v>
@@ -2117,7 +2117,7 @@
         <v>36</v>
       </c>
       <c r="C17" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D17" t="s">
         <v>38</v>
@@ -2129,13 +2129,13 @@
         <v>39</v>
       </c>
       <c r="G17" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H17" t="s">
+        <v>79</v>
+      </c>
+      <c r="I17" t="s">
         <v>80</v>
-      </c>
-      <c r="I17" t="s">
-        <v>81</v>
       </c>
       <c r="J17" t="s">
         <v>26</v>
@@ -2147,7 +2147,7 @@
         <v>100</v>
       </c>
       <c r="M17" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="N17" t="s">
         <v>34</v>
@@ -2215,13 +2215,13 @@
   <sheetData>
     <row r="1" spans="1:26" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>87</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -2245,22 +2245,22 @@
         <v>5</v>
       </c>
       <c r="K1" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>88</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>89</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="N1" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>92</v>
       </c>
       <c r="Q1" s="1" t="s">
         <v>12</v>
@@ -2269,10 +2269,10 @@
         <v>14</v>
       </c>
       <c r="S1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="T1" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>94</v>
       </c>
       <c r="U1" s="1" t="s">
         <v>15</v>
@@ -2281,10 +2281,10 @@
         <v>16</v>
       </c>
       <c r="W1" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="X1" s="1" t="s">
         <v>95</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>96</v>
       </c>
       <c r="Y1" s="1" t="s">
         <v>18</v>
@@ -2295,13 +2295,13 @@
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" t="s">
         <v>97</v>
-      </c>
-      <c r="B2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C2" t="s">
-        <v>98</v>
       </c>
       <c r="D2" t="s">
         <v>22</v>
@@ -2334,7 +2334,7 @@
         <v>40</v>
       </c>
       <c r="N2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="O2">
         <v>65</v>
@@ -2375,13 +2375,13 @@
     </row>
     <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B3" t="s">
         <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D3" t="s">
         <v>22</v>
@@ -2414,7 +2414,7 @@
         <v>40</v>
       </c>
       <c r="N3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O3">
         <v>65</v>
@@ -2455,13 +2455,13 @@
     </row>
     <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B4" t="s">
         <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D4" t="s">
         <v>22</v>
@@ -2494,7 +2494,7 @@
         <v>40</v>
       </c>
       <c r="N4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="O4">
         <v>65</v>
@@ -2535,13 +2535,13 @@
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B5" t="s">
         <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D5" t="s">
         <v>22</v>
@@ -2553,13 +2553,13 @@
         <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H5" t="s">
         <v>38</v>
       </c>
       <c r="I5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J5">
         <v>4</v>
@@ -2571,19 +2571,19 @@
         <v>23</v>
       </c>
       <c r="M5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O5">
         <v>100</v>
       </c>
       <c r="P5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="Q5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="R5" t="s">
         <v>44</v>
@@ -2615,13 +2615,13 @@
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B6" t="s">
         <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D6" t="s">
         <v>22</v>
@@ -2633,13 +2633,13 @@
         <v>36</v>
       </c>
       <c r="G6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="H6" t="s">
         <v>38</v>
       </c>
       <c r="I6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J6">
         <v>4</v>
@@ -2654,16 +2654,16 @@
         <v>40</v>
       </c>
       <c r="N6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="O6">
         <v>65</v>
       </c>
       <c r="P6" t="s">
+        <v>70</v>
+      </c>
+      <c r="Q6" t="s">
         <v>71</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>72</v>
       </c>
       <c r="R6" t="s">
         <v>44</v>
@@ -2695,13 +2695,13 @@
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B7" t="s">
         <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D7" t="s">
         <v>22</v>
@@ -2713,7 +2713,7 @@
         <v>36</v>
       </c>
       <c r="G7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H7" t="s">
         <v>38</v>
@@ -2731,19 +2731,19 @@
         <v>23</v>
       </c>
       <c r="M7" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="O7">
         <v>100</v>
       </c>
       <c r="P7" t="s">
+        <v>80</v>
+      </c>
+      <c r="Q7" t="s">
         <v>81</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>82</v>
       </c>
       <c r="R7" t="s">
         <v>44</v>
@@ -2775,31 +2775,31 @@
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B8" t="s">
         <v>23</v>
       </c>
       <c r="C8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D8" t="s">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="E8" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F8" t="s">
         <v>36</v>
       </c>
       <c r="G8" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="H8" t="s">
         <v>38</v>
       </c>
       <c r="I8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J8">
         <v>4</v>
@@ -2814,7 +2814,7 @@
         <v>49</v>
       </c>
       <c r="N8" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="O8">
         <v>150</v>
@@ -2823,7 +2823,7 @@
         <v>42</v>
       </c>
       <c r="Q8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="R8" t="s">
         <v>44</v>
@@ -2838,7 +2838,7 @@
         <v>45</v>
       </c>
       <c r="V8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="W8" t="s">
         <v>23</v>
@@ -2855,13 +2855,13 @@
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B9" t="s">
         <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D9" t="s">
         <v>31</v>
@@ -2894,7 +2894,7 @@
         <v>40</v>
       </c>
       <c r="N9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="O9">
         <v>65</v>
@@ -2935,13 +2935,13 @@
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B10" t="s">
         <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D10" t="s">
         <v>31</v>
@@ -2974,7 +2974,7 @@
         <v>40</v>
       </c>
       <c r="N10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="O10">
         <v>65</v>
@@ -3015,13 +3015,13 @@
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B11" t="s">
         <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D11" t="s">
         <v>31</v>
@@ -3033,13 +3033,13 @@
         <v>36</v>
       </c>
       <c r="G11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="H11" t="s">
         <v>38</v>
       </c>
       <c r="I11" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J11">
         <v>4</v>
@@ -3051,19 +3051,19 @@
         <v>23</v>
       </c>
       <c r="M11" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N11" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="O11">
         <v>100</v>
       </c>
       <c r="P11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="Q11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="R11" t="s">
         <v>44</v>
@@ -3095,13 +3095,13 @@
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B12" t="s">
         <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D12" t="s">
         <v>31</v>
@@ -3113,7 +3113,7 @@
         <v>36</v>
       </c>
       <c r="G12" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H12" t="s">
         <v>38</v>
@@ -3131,19 +3131,19 @@
         <v>23</v>
       </c>
       <c r="M12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N12" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="O12">
         <v>100</v>
       </c>
       <c r="P12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="Q12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="R12" t="s">
         <v>44</v>
@@ -3175,13 +3175,13 @@
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B13" t="s">
         <v>23</v>
       </c>
       <c r="C13" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D13" t="s">
         <v>47</v>
@@ -3214,7 +3214,7 @@
         <v>49</v>
       </c>
       <c r="N13" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="O13">
         <v>150</v>
@@ -3255,13 +3255,13 @@
     </row>
     <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B14" t="s">
         <v>23</v>
       </c>
       <c r="C14" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D14" t="s">
         <v>22</v>
@@ -3294,7 +3294,7 @@
         <v>40</v>
       </c>
       <c r="N14" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="O14">
         <v>65</v>
@@ -3351,7 +3351,7 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
@@ -3380,19 +3380,19 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>16</v>
@@ -3400,7 +3400,7 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B2" t="s">
         <v>28</v>
@@ -3409,7 +3409,7 @@
         <v>29</v>
       </c>
       <c r="D2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E2">
         <v>3</v>
@@ -3420,7 +3420,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B3" t="s">
         <v>34</v>
@@ -3472,70 +3472,70 @@
   <sheetData>
     <row r="1" spans="1:23" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>123</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>124</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>128</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>129</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>130</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>11</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="N1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>135</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="V1" s="1" t="s">
         <v>139</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>140</v>
       </c>
       <c r="W1" s="1" t="s">
         <v>16</v>
@@ -3543,82 +3543,82 @@
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B2" t="s">
         <v>141</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>142</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H2" t="s">
+        <v>23</v>
+      </c>
+      <c r="I2" t="s">
+        <v>23</v>
+      </c>
+      <c r="J2" t="s">
+        <v>23</v>
+      </c>
+      <c r="K2" t="s">
+        <v>23</v>
+      </c>
+      <c r="L2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M2" t="s">
         <v>143</v>
       </c>
-      <c r="D2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E2" t="s">
-        <v>23</v>
-      </c>
-      <c r="F2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G2" t="s">
-        <v>23</v>
-      </c>
-      <c r="H2" t="s">
-        <v>23</v>
-      </c>
-      <c r="I2" t="s">
-        <v>23</v>
-      </c>
-      <c r="J2" t="s">
-        <v>23</v>
-      </c>
-      <c r="K2" t="s">
-        <v>23</v>
-      </c>
-      <c r="L2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>23</v>
+      </c>
+      <c r="R2" t="s">
+        <v>23</v>
+      </c>
+      <c r="S2" t="s">
+        <v>23</v>
+      </c>
+      <c r="T2" t="s">
+        <v>23</v>
+      </c>
+      <c r="U2" t="s">
+        <v>23</v>
+      </c>
+      <c r="V2" t="s">
         <v>144</v>
       </c>
-      <c r="N2" t="s">
-        <v>23</v>
-      </c>
-      <c r="O2" t="s">
-        <v>23</v>
-      </c>
-      <c r="P2" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>23</v>
-      </c>
-      <c r="R2" t="s">
-        <v>23</v>
-      </c>
-      <c r="S2" t="s">
-        <v>23</v>
-      </c>
-      <c r="T2" t="s">
-        <v>23</v>
-      </c>
-      <c r="U2" t="s">
-        <v>23</v>
-      </c>
-      <c r="V2" t="s">
+      <c r="W2" t="s">
         <v>145</v>
-      </c>
-      <c r="W2" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B3" t="s">
         <v>141</v>
       </c>
-      <c r="B3" t="s">
-        <v>142</v>
-      </c>
       <c r="C3" t="s">
         <v>23</v>
       </c>
@@ -3641,16 +3641,16 @@
         <v>23</v>
       </c>
       <c r="J3" t="s">
+        <v>146</v>
+      </c>
+      <c r="K3" t="s">
         <v>147</v>
       </c>
-      <c r="K3" t="s">
-        <v>148</v>
-      </c>
       <c r="L3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="M3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="N3" t="s">
         <v>49</v>
@@ -3677,7 +3677,7 @@
         <v>23</v>
       </c>
       <c r="V3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="W3" t="s">
         <v>23</v>
@@ -3685,11 +3685,11 @@
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>140</v>
+      </c>
+      <c r="B4" t="s">
         <v>141</v>
       </c>
-      <c r="B4" t="s">
-        <v>142</v>
-      </c>
       <c r="C4" t="s">
         <v>23</v>
       </c>
@@ -3712,16 +3712,16 @@
         <v>23</v>
       </c>
       <c r="J4" t="s">
+        <v>146</v>
+      </c>
+      <c r="K4" t="s">
         <v>147</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>148</v>
       </c>
-      <c r="L4" t="s">
-        <v>149</v>
-      </c>
       <c r="M4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="N4" t="s">
         <v>49</v>
@@ -3748,7 +3748,7 @@
         <v>23</v>
       </c>
       <c r="V4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="W4" t="s">
         <v>23</v>
@@ -3756,22 +3756,22 @@
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>149</v>
+      </c>
+      <c r="B5" t="s">
         <v>150</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>151</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" t="s">
         <v>152</v>
-      </c>
-      <c r="D5" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" t="s">
-        <v>153</v>
       </c>
       <c r="G5" t="s">
         <v>23</v>
@@ -3819,21 +3819,21 @@
         <v>23</v>
       </c>
       <c r="V5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="W5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>149</v>
+      </c>
+      <c r="B6" t="s">
         <v>150</v>
       </c>
-      <c r="B6" t="s">
-        <v>151</v>
-      </c>
       <c r="C6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D6" t="s">
         <v>23</v>
@@ -3842,7 +3842,7 @@
         <v>23</v>
       </c>
       <c r="F6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G6" t="s">
         <v>23</v>
@@ -3890,7 +3890,7 @@
         <v>23</v>
       </c>
       <c r="V6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="W6" t="s">
         <v>23</v>
@@ -3898,13 +3898,13 @@
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>149</v>
+      </c>
+      <c r="B7" t="s">
         <v>150</v>
       </c>
-      <c r="B7" t="s">
-        <v>151</v>
-      </c>
       <c r="C7" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D7" t="s">
         <v>23</v>
@@ -3913,7 +3913,7 @@
         <v>23</v>
       </c>
       <c r="F7" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G7" t="s">
         <v>23</v>
@@ -3961,7 +3961,7 @@
         <v>23</v>
       </c>
       <c r="V7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="W7" t="s">
         <v>23</v>
@@ -3969,13 +3969,13 @@
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B8" t="s">
         <v>150</v>
       </c>
-      <c r="B8" t="s">
-        <v>151</v>
-      </c>
       <c r="C8" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D8" t="s">
         <v>23</v>
@@ -3984,7 +3984,7 @@
         <v>23</v>
       </c>
       <c r="F8" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G8" t="s">
         <v>23</v>
@@ -4032,7 +4032,7 @@
         <v>23</v>
       </c>
       <c r="V8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="W8" t="s">
         <v>23</v>
@@ -4040,13 +4040,13 @@
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>149</v>
+      </c>
+      <c r="B9" t="s">
         <v>150</v>
       </c>
-      <c r="B9" t="s">
-        <v>151</v>
-      </c>
       <c r="C9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D9" t="s">
         <v>23</v>
@@ -4055,7 +4055,7 @@
         <v>23</v>
       </c>
       <c r="F9" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G9" t="s">
         <v>23</v>
@@ -4103,7 +4103,7 @@
         <v>23</v>
       </c>
       <c r="V9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="W9" t="s">
         <v>23</v>
@@ -4111,13 +4111,13 @@
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>149</v>
+      </c>
+      <c r="B10" t="s">
         <v>150</v>
       </c>
-      <c r="B10" t="s">
-        <v>151</v>
-      </c>
       <c r="C10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D10" t="s">
         <v>23</v>
@@ -4126,7 +4126,7 @@
         <v>23</v>
       </c>
       <c r="F10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G10" t="s">
         <v>23</v>
@@ -4174,7 +4174,7 @@
         <v>23</v>
       </c>
       <c r="V10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="W10" t="s">
         <v>23</v>
@@ -4182,13 +4182,13 @@
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>149</v>
+      </c>
+      <c r="B11" t="s">
         <v>150</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>151</v>
-      </c>
-      <c r="C11" t="s">
-        <v>152</v>
       </c>
       <c r="D11" t="s">
         <v>23</v>
@@ -4242,10 +4242,10 @@
         <v>23</v>
       </c>
       <c r="U11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="V11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="W11" t="s">
         <v>23</v>
@@ -4253,13 +4253,13 @@
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>149</v>
+      </c>
+      <c r="B12" t="s">
         <v>150</v>
       </c>
-      <c r="B12" t="s">
-        <v>151</v>
-      </c>
       <c r="C12" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D12" t="s">
         <v>23</v>
@@ -4313,10 +4313,10 @@
         <v>23</v>
       </c>
       <c r="U12" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="V12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="W12" t="s">
         <v>23</v>
@@ -4324,13 +4324,13 @@
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>149</v>
+      </c>
+      <c r="B13" t="s">
         <v>150</v>
       </c>
-      <c r="B13" t="s">
-        <v>151</v>
-      </c>
       <c r="C13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D13" t="s">
         <v>23</v>
@@ -4384,10 +4384,10 @@
         <v>23</v>
       </c>
       <c r="U13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="V13" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="W13" t="s">
         <v>23</v>
@@ -4395,13 +4395,13 @@
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>149</v>
+      </c>
+      <c r="B14" t="s">
         <v>150</v>
       </c>
-      <c r="B14" t="s">
-        <v>151</v>
-      </c>
       <c r="C14" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D14" t="s">
         <v>23</v>
@@ -4455,10 +4455,10 @@
         <v>23</v>
       </c>
       <c r="U14" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="V14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="W14" t="s">
         <v>23</v>
@@ -4483,27 +4483,27 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>159</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>160</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>161</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>162</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B2" t="s">
         <v>22</v>
@@ -4523,7 +4523,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B3" t="s">
         <v>31</v>
@@ -4543,10 +4543,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>164</v>
+      </c>
+      <c r="B4" t="s">
         <v>165</v>
-      </c>
-      <c r="B4" t="s">
-        <v>166</v>
       </c>
       <c r="C4" t="s">
         <v>23</v>
@@ -4563,10 +4563,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C5" t="s">
         <v>23</v>
@@ -4583,10 +4583,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C6" t="s">
         <v>23</v>
@@ -4609,7 +4609,7 @@
         <v>22</v>
       </c>
       <c r="C7" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D7" t="s">
         <v>23</v>
@@ -4626,7 +4626,7 @@
         <v>0</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>169</v>
       </c>
       <c r="C8" t="s">
         <v>170</v>
@@ -4832,7 +4832,7 @@
         <v>185</v>
       </c>
       <c r="D18" t="s">
-        <v>63</v>
+        <v>169</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -4885,12 +4885,12 @@
         <v>192</v>
       </c>
       <c r="B4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B5" t="s">
         <v>23</v>
@@ -4917,7 +4917,7 @@
         <v>196</v>
       </c>
       <c r="B8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Cohort examples count the students outside the cohort
The Merging schedules example's cohort rule and the user guide's cohort example
each add the other students who take one of the courses on its own, as groups of
their own with that one course, with seats to match. Merged, the example's rule
is short by one student (87 of 88) and its advice still fixes it. The guide's
Examples list now points to Merging schedules for cohort planning.

Assisted by Claude Opus 5.5 (Anthropic).
</commit_message>
<xml_diff>
--- a/apps/web/public/examples/example-merging-amus.xlsx
+++ b/apps/web/public/examples/example-merging-amus.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1141" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1233" uniqueCount="208">
   <si>
     <t>Term</t>
   </si>
@@ -478,7 +478,7 @@
     <t>30</t>
   </si>
   <si>
-    <t>Two groups of 30 first-year students who share BHAV 112 and DIGI 225. The courses are in three schedules, so the rule can only be checked when they are merged.</t>
+    <t>Two groups of 30 first-year students who share BHAV 112 and DIGI 225, and the other students who take one of the courses on its own (groups 3 to 6). The courses are in three schedules, so the rule can only be checked when they are merged.</t>
   </si>
   <si>
     <t>BHAV 112</t>
@@ -490,9 +490,33 @@
     <t>AMUS 145</t>
   </si>
   <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
     <t>25</t>
   </si>
   <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>34</t>
+  </si>
+  <si>
     <t>Kind</t>
   </si>
   <si>
@@ -586,13 +610,13 @@
     <t>Export Date</t>
   </si>
   <si>
-    <t>2026-10-07</t>
+    <t>2026-10-11</t>
   </si>
   <si>
     <t>Export Time</t>
   </si>
   <si>
-    <t>15:09:00</t>
+    <t>14:44:40</t>
   </si>
   <si>
     <t>Academic Year</t>
@@ -3446,7 +3470,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W14"/>
+  <dimension ref="A1:W18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -4197,7 +4221,7 @@
         <v>23</v>
       </c>
       <c r="F11" t="s">
-        <v>23</v>
+        <v>157</v>
       </c>
       <c r="G11" t="s">
         <v>23</v>
@@ -4239,10 +4263,10 @@
         <v>23</v>
       </c>
       <c r="T11" t="s">
-        <v>23</v>
+        <v>158</v>
       </c>
       <c r="U11" t="s">
-        <v>157</v>
+        <v>23</v>
       </c>
       <c r="V11" t="s">
         <v>144</v>
@@ -4268,7 +4292,7 @@
         <v>23</v>
       </c>
       <c r="F12" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="G12" t="s">
         <v>23</v>
@@ -4310,10 +4334,10 @@
         <v>23</v>
       </c>
       <c r="T12" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="U12" t="s">
-        <v>157</v>
+        <v>23</v>
       </c>
       <c r="V12" t="s">
         <v>144</v>
@@ -4339,7 +4363,7 @@
         <v>23</v>
       </c>
       <c r="F13" t="s">
-        <v>23</v>
+        <v>159</v>
       </c>
       <c r="G13" t="s">
         <v>23</v>
@@ -4381,10 +4405,10 @@
         <v>23</v>
       </c>
       <c r="T13" t="s">
-        <v>23</v>
+        <v>160</v>
       </c>
       <c r="U13" t="s">
-        <v>152</v>
+        <v>23</v>
       </c>
       <c r="V13" t="s">
         <v>144</v>
@@ -4410,7 +4434,7 @@
         <v>23</v>
       </c>
       <c r="F14" t="s">
-        <v>23</v>
+        <v>161</v>
       </c>
       <c r="G14" t="s">
         <v>23</v>
@@ -4452,15 +4476,299 @@
         <v>23</v>
       </c>
       <c r="T14" t="s">
-        <v>23</v>
+        <v>157</v>
       </c>
       <c r="U14" t="s">
-        <v>152</v>
+        <v>23</v>
       </c>
       <c r="V14" t="s">
         <v>144</v>
       </c>
       <c r="W14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>149</v>
+      </c>
+      <c r="B15" t="s">
+        <v>150</v>
+      </c>
+      <c r="C15" t="s">
+        <v>151</v>
+      </c>
+      <c r="D15" t="s">
+        <v>23</v>
+      </c>
+      <c r="E15" t="s">
+        <v>23</v>
+      </c>
+      <c r="F15" t="s">
+        <v>23</v>
+      </c>
+      <c r="G15" t="s">
+        <v>23</v>
+      </c>
+      <c r="H15" t="s">
+        <v>23</v>
+      </c>
+      <c r="I15" t="s">
+        <v>23</v>
+      </c>
+      <c r="J15" t="s">
+        <v>23</v>
+      </c>
+      <c r="K15" t="s">
+        <v>23</v>
+      </c>
+      <c r="L15" t="s">
+        <v>23</v>
+      </c>
+      <c r="M15" t="s">
+        <v>22</v>
+      </c>
+      <c r="N15" t="s">
+        <v>23</v>
+      </c>
+      <c r="O15" t="s">
+        <v>23</v>
+      </c>
+      <c r="P15" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>23</v>
+      </c>
+      <c r="R15" t="s">
+        <v>23</v>
+      </c>
+      <c r="S15" t="s">
+        <v>23</v>
+      </c>
+      <c r="T15" t="s">
+        <v>23</v>
+      </c>
+      <c r="U15" t="s">
+        <v>162</v>
+      </c>
+      <c r="V15" t="s">
+        <v>144</v>
+      </c>
+      <c r="W15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>149</v>
+      </c>
+      <c r="B16" t="s">
+        <v>150</v>
+      </c>
+      <c r="C16" t="s">
+        <v>156</v>
+      </c>
+      <c r="D16" t="s">
+        <v>23</v>
+      </c>
+      <c r="E16" t="s">
+        <v>23</v>
+      </c>
+      <c r="F16" t="s">
+        <v>23</v>
+      </c>
+      <c r="G16" t="s">
+        <v>23</v>
+      </c>
+      <c r="H16" t="s">
+        <v>23</v>
+      </c>
+      <c r="I16" t="s">
+        <v>23</v>
+      </c>
+      <c r="J16" t="s">
+        <v>23</v>
+      </c>
+      <c r="K16" t="s">
+        <v>23</v>
+      </c>
+      <c r="L16" t="s">
+        <v>23</v>
+      </c>
+      <c r="M16" t="s">
+        <v>22</v>
+      </c>
+      <c r="N16" t="s">
+        <v>23</v>
+      </c>
+      <c r="O16" t="s">
+        <v>23</v>
+      </c>
+      <c r="P16" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>23</v>
+      </c>
+      <c r="R16" t="s">
+        <v>23</v>
+      </c>
+      <c r="S16" t="s">
+        <v>23</v>
+      </c>
+      <c r="T16" t="s">
+        <v>23</v>
+      </c>
+      <c r="U16" t="s">
+        <v>163</v>
+      </c>
+      <c r="V16" t="s">
+        <v>144</v>
+      </c>
+      <c r="W16" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>149</v>
+      </c>
+      <c r="B17" t="s">
+        <v>150</v>
+      </c>
+      <c r="C17" t="s">
+        <v>154</v>
+      </c>
+      <c r="D17" t="s">
+        <v>23</v>
+      </c>
+      <c r="E17" t="s">
+        <v>23</v>
+      </c>
+      <c r="F17" t="s">
+        <v>23</v>
+      </c>
+      <c r="G17" t="s">
+        <v>23</v>
+      </c>
+      <c r="H17" t="s">
+        <v>23</v>
+      </c>
+      <c r="I17" t="s">
+        <v>23</v>
+      </c>
+      <c r="J17" t="s">
+        <v>23</v>
+      </c>
+      <c r="K17" t="s">
+        <v>23</v>
+      </c>
+      <c r="L17" t="s">
+        <v>23</v>
+      </c>
+      <c r="M17" t="s">
+        <v>22</v>
+      </c>
+      <c r="N17" t="s">
+        <v>23</v>
+      </c>
+      <c r="O17" t="s">
+        <v>23</v>
+      </c>
+      <c r="P17" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q17" t="s">
+        <v>23</v>
+      </c>
+      <c r="R17" t="s">
+        <v>23</v>
+      </c>
+      <c r="S17" t="s">
+        <v>23</v>
+      </c>
+      <c r="T17" t="s">
+        <v>23</v>
+      </c>
+      <c r="U17" t="s">
+        <v>164</v>
+      </c>
+      <c r="V17" t="s">
+        <v>144</v>
+      </c>
+      <c r="W17" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>149</v>
+      </c>
+      <c r="B18" t="s">
+        <v>150</v>
+      </c>
+      <c r="C18" t="s">
+        <v>155</v>
+      </c>
+      <c r="D18" t="s">
+        <v>23</v>
+      </c>
+      <c r="E18" t="s">
+        <v>23</v>
+      </c>
+      <c r="F18" t="s">
+        <v>23</v>
+      </c>
+      <c r="G18" t="s">
+        <v>23</v>
+      </c>
+      <c r="H18" t="s">
+        <v>23</v>
+      </c>
+      <c r="I18" t="s">
+        <v>23</v>
+      </c>
+      <c r="J18" t="s">
+        <v>23</v>
+      </c>
+      <c r="K18" t="s">
+        <v>23</v>
+      </c>
+      <c r="L18" t="s">
+        <v>23</v>
+      </c>
+      <c r="M18" t="s">
+        <v>22</v>
+      </c>
+      <c r="N18" t="s">
+        <v>23</v>
+      </c>
+      <c r="O18" t="s">
+        <v>23</v>
+      </c>
+      <c r="P18" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>23</v>
+      </c>
+      <c r="R18" t="s">
+        <v>23</v>
+      </c>
+      <c r="S18" t="s">
+        <v>23</v>
+      </c>
+      <c r="T18" t="s">
+        <v>23</v>
+      </c>
+      <c r="U18" t="s">
+        <v>165</v>
+      </c>
+      <c r="V18" t="s">
+        <v>144</v>
+      </c>
+      <c r="W18" t="s">
         <v>23</v>
       </c>
     </row>
@@ -4483,27 +4791,27 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="B2" t="s">
         <v>22</v>
@@ -4523,7 +4831,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="B3" t="s">
         <v>31</v>
@@ -4543,10 +4851,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="C4" t="s">
         <v>23</v>
@@ -4563,10 +4871,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="B5" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="C5" t="s">
         <v>23</v>
@@ -4583,10 +4891,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="B6" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="C6" t="s">
         <v>23</v>
@@ -4609,7 +4917,7 @@
         <v>22</v>
       </c>
       <c r="C7" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="D7" t="s">
         <v>23</v>
@@ -4626,10 +4934,10 @@
         <v>0</v>
       </c>
       <c r="B8" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="C8" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="D8" t="s">
         <v>23</v>
@@ -4649,7 +4957,7 @@
         <v>31</v>
       </c>
       <c r="C9" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="D9" t="s">
         <v>23</v>
@@ -4669,7 +4977,7 @@
         <v>47</v>
       </c>
       <c r="C10" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="D10" t="s">
         <v>23</v>
@@ -4683,13 +4991,13 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B11" t="s">
         <v>26</v>
       </c>
       <c r="C11" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="D11" t="s">
         <v>23</v>
@@ -4703,13 +5011,13 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B12" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="C12" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="D12" t="s">
         <v>23</v>
@@ -4723,13 +5031,13 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B13" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="C13" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="D13" t="s">
         <v>23</v>
@@ -4743,13 +5051,13 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B14" t="s">
         <v>38</v>
       </c>
       <c r="C14" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="D14" t="s">
         <v>23</v>
@@ -4763,13 +5071,13 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B15" t="s">
         <v>53</v>
       </c>
       <c r="C15" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="D15" t="s">
         <v>23</v>
@@ -4783,13 +5091,13 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B16" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="C16" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="D16" t="s">
         <v>23</v>
@@ -4803,13 +5111,13 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B17" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="C17" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="D17" t="s">
         <v>23</v>
@@ -4823,16 +5131,16 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="B18" t="s">
         <v>26</v>
       </c>
       <c r="C18" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="D18" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -4858,31 +5166,31 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="B2" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="B3" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="B4" t="s">
         <v>97</v>
@@ -4890,7 +5198,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B5" t="s">
         <v>23</v>
@@ -4898,7 +5206,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="B6" t="s">
         <v>23</v>
@@ -4906,15 +5214,15 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="B7" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="B8" t="s">
         <v>144</v>
@@ -4922,7 +5230,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="B9" t="s">
         <v>23</v>
@@ -4930,7 +5238,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="B10" t="s">
         <v>23</v>
@@ -4938,7 +5246,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="B11" t="s">
         <v>23</v>

</xml_diff>

<commit_message>
Example "Merging schedules/cohort planning": enough seats, but the times keep 6 of 98 students out
Renamed from "Merging schedules". The cohort rule now has two groups of 40 and
a few students outside the cohort in each course, with enough seats in every
course; merged, the clash of DIGI 225 B and AMUS 145 B with BHAV 112 A leaves
92 of 98 seated, and moving DIGI 225 B to another time seats everyone (the
example's test checks both).

Assisted by Claude Opus 5.5 (Anthropic).
</commit_message>
<xml_diff>
--- a/apps/web/public/examples/example-merging-amus.xlsx
+++ b/apps/web/public/examples/example-merging-amus.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1233" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1233" uniqueCount="204">
   <si>
     <t>Term</t>
   </si>
@@ -475,10 +475,10 @@
     <t>AMUS 112</t>
   </si>
   <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>Two groups of 30 first-year students who share BHAV 112 and DIGI 225, and the other students who take one of the courses on its own (groups 3 to 6). The courses are in three schedules, so the rule can only be checked when they are merged.</t>
+    <t>40</t>
+  </si>
+  <si>
+    <t>Two groups of 40 first-year students who share BHAV 112 and DIGI 225, and the other students who take one of the courses on its own (groups 3 to 6). The courses are in three schedules, so the rule can only be checked when they are merged.</t>
   </si>
   <si>
     <t>BHAV 112</t>
@@ -496,25 +496,13 @@
     <t>3</t>
   </si>
   <si>
-    <t>10</t>
-  </si>
-  <si>
     <t>5</t>
   </si>
   <si>
-    <t>8</t>
-  </si>
-  <si>
     <t>25</t>
   </si>
   <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>35</t>
-  </si>
-  <si>
-    <t>34</t>
+    <t>42</t>
   </si>
   <si>
     <t>Kind</t>
@@ -616,7 +604,7 @@
     <t>Export Time</t>
   </si>
   <si>
-    <t>14:44:40</t>
+    <t>15:16:14</t>
   </si>
   <si>
     <t>Academic Year</t>
@@ -4363,7 +4351,7 @@
         <v>23</v>
       </c>
       <c r="F13" t="s">
-        <v>159</v>
+        <v>39</v>
       </c>
       <c r="G13" t="s">
         <v>23</v>
@@ -4405,7 +4393,7 @@
         <v>23</v>
       </c>
       <c r="T13" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="U13" t="s">
         <v>23</v>
@@ -4434,7 +4422,7 @@
         <v>23</v>
       </c>
       <c r="F14" t="s">
-        <v>161</v>
+        <v>39</v>
       </c>
       <c r="G14" t="s">
         <v>23</v>
@@ -4550,7 +4538,7 @@
         <v>23</v>
       </c>
       <c r="U15" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="V15" t="s">
         <v>144</v>
@@ -4621,7 +4609,7 @@
         <v>23</v>
       </c>
       <c r="U16" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="V16" t="s">
         <v>144</v>
@@ -4692,7 +4680,7 @@
         <v>23</v>
       </c>
       <c r="U17" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="V17" t="s">
         <v>144</v>
@@ -4763,7 +4751,7 @@
         <v>23</v>
       </c>
       <c r="U18" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="V18" t="s">
         <v>144</v>
@@ -4791,27 +4779,27 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B2" t="s">
         <v>22</v>
@@ -4831,7 +4819,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B3" t="s">
         <v>31</v>
@@ -4851,10 +4839,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="C4" t="s">
         <v>23</v>
@@ -4871,10 +4859,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B5" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="C5" t="s">
         <v>23</v>
@@ -4891,10 +4879,10 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B6" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C6" t="s">
         <v>23</v>
@@ -4917,7 +4905,7 @@
         <v>22</v>
       </c>
       <c r="C7" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="D7" t="s">
         <v>23</v>
@@ -4934,10 +4922,10 @@
         <v>0</v>
       </c>
       <c r="B8" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="C8" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D8" t="s">
         <v>23</v>
@@ -4957,7 +4945,7 @@
         <v>31</v>
       </c>
       <c r="C9" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D9" t="s">
         <v>23</v>
@@ -4977,7 +4965,7 @@
         <v>47</v>
       </c>
       <c r="C10" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="D10" t="s">
         <v>23</v>
@@ -4991,13 +4979,13 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B11" t="s">
         <v>26</v>
       </c>
       <c r="C11" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="D11" t="s">
         <v>23</v>
@@ -5011,13 +4999,13 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B12" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="C12" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D12" t="s">
         <v>23</v>
@@ -5031,13 +5019,13 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>177</v>
+      </c>
+      <c r="B13" t="s">
         <v>181</v>
       </c>
-      <c r="B13" t="s">
-        <v>185</v>
-      </c>
       <c r="C13" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="D13" t="s">
         <v>23</v>
@@ -5051,13 +5039,13 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B14" t="s">
         <v>38</v>
       </c>
       <c r="C14" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="D14" t="s">
         <v>23</v>
@@ -5071,13 +5059,13 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B15" t="s">
         <v>53</v>
       </c>
       <c r="C15" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="D15" t="s">
         <v>23</v>
@@ -5091,13 +5079,13 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B16" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="C16" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="D16" t="s">
         <v>23</v>
@@ -5111,13 +5099,13 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B17" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C17" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="D17" t="s">
         <v>23</v>
@@ -5131,16 +5119,16 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B18" t="s">
         <v>26</v>
       </c>
       <c r="C18" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="D18" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="E18">
         <v>1</v>
@@ -5166,31 +5154,31 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B2" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B3" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="B4" t="s">
         <v>97</v>
@@ -5198,7 +5186,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B5" t="s">
         <v>23</v>
@@ -5206,7 +5194,7 @@
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="B6" t="s">
         <v>23</v>
@@ -5214,15 +5202,15 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B7" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="B8" t="s">
         <v>144</v>
@@ -5230,7 +5218,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B9" t="s">
         <v>23</v>
@@ -5238,7 +5226,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B10" t="s">
         <v>23</v>
@@ -5246,7 +5234,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="B11" t="s">
         <v>23</v>

</xml_diff>